<commit_message>
Added more calibration plot data.
</commit_message>
<xml_diff>
--- a/calibration_plots/plot_data_glass_mpbart.xlsx
+++ b/calibration_plots/plot_data_glass_mpbart.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -368,50 +368,42 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>0.3954814814814815</v>
+        <v>0.4068682170542636</v>
       </c>
       <c r="B2">
-        <v>0.4722222222222222</v>
+        <v>0.5348837209302325</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>0.5002962962962962</v>
+        <v>0.5194418604651163</v>
       </c>
       <c r="B3">
-        <v>0.5833333333333334</v>
+        <v>0.5581395348837209</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>0.5565523809523809</v>
+        <v>0.5936349206349206</v>
       </c>
       <c r="B4">
-        <v>0.6857142857142857</v>
+        <v>0.7857142857142857</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>0.638537037037037</v>
+        <v>0.7076434108527132</v>
       </c>
       <c r="B5">
-        <v>0.8333333333333334</v>
+        <v>0.8604651162790697</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>0.7403238095238095</v>
+        <v>0.8347751937984496</v>
       </c>
       <c r="B6">
-        <v>0.8571428571428571</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>0.8461666666666666</v>
-      </c>
-      <c r="B7">
-        <v>0.8611111111111112</v>
+        <v>0.8372093023255814</v>
       </c>
     </row>
   </sheetData>

</xml_diff>